<commit_message>
[Issue #2] update archive log with PR number
</commit_message>
<xml_diff>
--- a/commits-log.xlsx
+++ b/commits-log.xlsx
@@ -1,202 +1,285 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="25600" windowHeight="12200" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView windowWidth="25600" windowHeight="12200"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug__" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Bug__" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+  <si>
+    <t>Issue</t>
+  </si>
+  <si>
+    <t>PR</t>
+  </si>
+  <si>
+    <t>阶段</t>
+  </si>
+  <si>
+    <t>分支</t>
+  </si>
+  <si>
+    <t>测试文件</t>
+  </si>
+  <si>
+    <t>修复文件</t>
+  </si>
+  <si>
+    <t>关键 Commit</t>
+  </si>
+  <si>
+    <t>状态</t>
+  </si>
+  <si>
+    <t>#1</t>
+  </si>
+  <si>
+    <t>#3</t>
+  </si>
+  <si>
+    <t>后期</t>
+  </si>
+  <si>
+    <t>fix/issue-001-f28-global-call-stack-slot</t>
+  </si>
+  <si>
+    <t>tests/integration/test_abc_pipeline.cpp</t>
+  </si>
+  <si>
+    <t>src/backend/register_allocator.cpp</t>
+  </si>
+  <si>
+    <t>121f04a; 3d2e73a</t>
+  </si>
+  <si>
+    <t>已合入</t>
+  </si>
+  <si>
+    <t>#2</t>
+  </si>
+  <si>
+    <t>#4</t>
+  </si>
+  <si>
+    <t>中期</t>
+  </si>
+  <si>
+    <t>fix/issue-002-icmp-eq-codegen</t>
+  </si>
+  <si>
+    <t>src/backend/code_generator.cpp</t>
+  </si>
+  <si>
+    <t>3989195; 1861864</t>
+  </si>
+  <si>
+    <t>待创建PR/待合入</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="25">
-    <font>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="23">
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <sz val="11"/>
-    </font>
-    <font>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="宋体"/>
       <charset val="134"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
-      <sz val="11"/>
-    </font>
-    <font>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <color rgb="FF0000FF"/>
-      <sz val="11"/>
-      <u val="single"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <color rgb="FF800080"/>
-      <sz val="11"/>
-      <u val="single"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <color rgb="FFFF0000"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="18"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <i val="1"/>
-      <color rgb="FF7F7F7F"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="15"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="13"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <color rgb="FF3F3F76"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <b val="1"/>
-      <color rgb="FF3F3F3F"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <b val="1"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <b val="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <color rgb="FF006100"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <color rgb="FF9C0006"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <color rgb="FF9C6500"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <color theme="0"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="33">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -496,165 +579,163 @@
     </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="6" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -900,7 +981,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
       <tableStyleElement type="wholeTable" dxfId="6"/>
       <tableStyleElement type="headerRow" dxfId="5"/>
       <tableStyleElement type="totalRow" dxfId="4"/>
@@ -909,7 +990,7 @@
       <tableStyleElement type="firstRowStripe" dxfId="1"/>
       <tableStyleElement type="firstColumnStripe" dxfId="0"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10">
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
       <tableStyleElement type="headerRow" dxfId="16"/>
       <tableStyleElement type="totalRow" dxfId="15"/>
       <tableStyleElement type="firstRowStripe" dxfId="14"/>
@@ -922,74 +1003,11 @@
       <tableStyleElement type="pageFieldValues" dxfId="7"/>
     </tableStyle>
   </tableStyles>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -1249,151 +1267,100 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:H3"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9.81818181818182" defaultRowHeight="14.5" outlineLevelRow="1"/>
+  <sheetFormatPr defaultColWidth="9.81818181818182" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="7"/>
   <cols>
-    <col width="10" customWidth="1" style="4" min="1" max="1"/>
-    <col width="28" customWidth="1" style="4" min="2" max="2"/>
-    <col width="10" customWidth="1" style="4" min="3" max="3"/>
-    <col width="42" customWidth="1" style="4" min="4" max="5"/>
-    <col width="42" customWidth="1" style="4" min="5" max="5"/>
-    <col width="36" customWidth="1" style="4" min="6" max="6"/>
-    <col width="24" customWidth="1" style="4" min="7" max="7"/>
-    <col width="20" customWidth="1" style="4" min="8" max="8"/>
+    <col min="1" max="1" width="10" style="1" customWidth="1"/>
+    <col min="2" max="2" width="28" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10" style="1" customWidth="1"/>
+    <col min="4" max="5" width="42" style="1" customWidth="1"/>
+    <col min="6" max="6" width="36" style="1" customWidth="1"/>
+    <col min="7" max="7" width="24" style="1" customWidth="1"/>
+    <col min="8" max="8" width="20" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>Issue</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>PR</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>阶段</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>分支</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>测试文件</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>修复文件</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>关键 Commit</t>
-        </is>
-      </c>
-      <c r="H1" s="5" t="inlineStr">
-        <is>
-          <t>状态</t>
-        </is>
+    <row r="1" spans="1:8">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="0" t="inlineStr">
-        <is>
-          <t>#1</t>
-        </is>
-      </c>
-      <c r="B2" s="0" t="inlineStr">
-        <is>
-          <t>#3</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>后期</t>
-        </is>
-      </c>
-      <c r="D2" s="0" t="inlineStr">
-        <is>
-          <t>fix/issue-001-f28-global-call-stack-slot</t>
-        </is>
-      </c>
-      <c r="E2" s="0" t="inlineStr">
-        <is>
-          <t>tests/integration/test_abc_pipeline.cpp</t>
-        </is>
-      </c>
-      <c r="F2" s="0" t="inlineStr">
-        <is>
-          <t>src/backend/register_allocator.cpp</t>
-        </is>
-      </c>
-      <c r="G2" s="0" t="inlineStr">
-        <is>
-          <t>121f04a; 3d2e73a</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>已合入</t>
-        </is>
+    <row r="2" spans="1:8">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>15</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="0" t="inlineStr">
-        <is>
-          <t>#2</t>
-        </is>
-      </c>
-      <c r="B3" s="0" t="inlineStr">
-        <is>
-          <t>待补充（PR创建后填写）</t>
-        </is>
-      </c>
-      <c r="C3" s="0" t="inlineStr">
-        <is>
-          <t>中期</t>
-        </is>
-      </c>
-      <c r="D3" s="0" t="inlineStr">
-        <is>
-          <t>fix/issue-002-icmp-eq-codegen</t>
-        </is>
-      </c>
-      <c r="E3" s="0" t="inlineStr">
-        <is>
-          <t>tests/integration/test_abc_pipeline.cpp</t>
-        </is>
-      </c>
-      <c r="F3" s="0" t="inlineStr">
-        <is>
-          <t>src/backend/code_generator.cpp</t>
-        </is>
-      </c>
-      <c r="G3" s="0" t="inlineStr">
-        <is>
-          <t>3989195; 1861864</t>
-        </is>
-      </c>
-      <c r="H3" s="0" t="inlineStr">
-        <is>
-          <t>待创建PR/待合入</t>
-        </is>
+    <row r="3" spans="1:8">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>